<commit_message>
feat(skills): update lifecycle skills to v3.11.0, sync anti-code leak rules and manifest
</commit_message>
<xml_diff>
--- a/skills/a7-estimate-template-fill/assets/MPL-H12 App_IOS_見積書_template.xlsx
+++ b/skills/a7-estimate-template-fill/assets/MPL-H12 App_IOS_見積書_template.xlsx
@@ -31,75 +31,19 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="308">
   <si>
-    <t xml:space="preserve">株式会社リッケイ</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="DejaVu Sans"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">〒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">108-0023 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="DejaVu Sans"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">東京都港区芝浦</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">3-1-21 msb Tamachi </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="DejaVu Sans"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">田町ステーションタワー</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">S 10F</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Tel: 03 6435 0754</t>
+    <t xml:space="preserve">システム開発受託チーム</t>
+  </si>
+  <si>
+    <t xml:space="preserve">〒100-0001 東京都千代田区千代田1-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03-1234-5678</t>
   </si>
   <si>
     <t xml:space="preserve">御見積書</t>
   </si>
   <si>
-    <t xml:space="preserve">MPL-H12 App_IOS</t>
+    <t xml:space="preserve">法人向け契約・請求・入金管理システム</t>
   </si>
   <si>
     <t xml:space="preserve">バージョン</t>
@@ -114,7 +58,7 @@
     <t xml:space="preserve">変更内容</t>
   </si>
   <si>
-    <t xml:space="preserve">リッケイ</t>
+    <t xml:space="preserve">開発元</t>
   </si>
   <si>
     <t xml:space="preserve">新規作成</t>
@@ -182,7 +126,7 @@
         <family val="2"/>
         <charset val="128"/>
       </rPr>
-      <t xml:space="preserve">20231013Rikkei</t>
+      <t xml:space="preserve">20231013</t>
     </r>
     <r>
       <rPr>
@@ -1952,7 +1896,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">yêu cầu của khách hàng</t>
+    <t xml:space="preserve">お客様要件仕様書・要求事項</t>
   </si>
   <si>
     <r>
@@ -2021,13 +1965,13 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Hạng mục</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phương pháp thực hiện</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ghi chú</t>
+    <t xml:space="preserve">項目</t>
+  </si>
+  <si>
+    <t xml:space="preserve">実施方式・対応方針</t>
+  </si>
+  <si>
+    <t xml:space="preserve">備考</t>
   </si>
   <si>
     <r>
@@ -2063,13 +2007,13 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Hạng mục test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nội dung xác nhận</t>
-  </si>
-  <si>
-    <t xml:space="preserve">※Nếu có yêu cầu test trên nhiều môi trường hoặc thêm test case ngoài phạm vi trên, effort test sẽ được xem xét và báo giá lại.</t>
+    <t xml:space="preserve">テスト項目</t>
+  </si>
+  <si>
+    <t xml:space="preserve">確認内容</t>
+  </si>
+  <si>
+    <t xml:space="preserve">※複数環境での検証や上記スコープ外のテストケース追加が必要な場合は、別途テスト工数を精算・再見積りいたします。</t>
   </si>
   <si>
     <r>
@@ -2211,7 +2155,7 @@
     <t xml:space="preserve">受入テスト</t>
   </si>
   <si>
-    <t xml:space="preserve">リッケイの対応</t>
+    <t xml:space="preserve">開発元の対応</t>
   </si>
   <si>
     <r>
@@ -2231,7 +2175,7 @@
         <rFont val="DejaVu Sans"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">様がテスト実施、リッケイが指摘より対応</t>
+      <t xml:space="preserve">様がテスト実施、開発元が指摘より対応</t>
     </r>
   </si>
   <si>
@@ -2301,34 +2245,16 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="DejaVu Sans"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">・</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">Các tài liệu/cấu hình dưới đây được dự kiến là deliverables của phạm vi này.</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">■Danh sách deliverables</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tên deliverable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mô tả</t>
+    <t xml:space="preserve">本スコープにおける納品成果物（ドキュメントおよび設定一式）は以下の通りです。</t>
+  </si>
+  <si>
+    <t xml:space="preserve">■納品成果物一覧</t>
+  </si>
+  <si>
+    <t xml:space="preserve">成果物名称</t>
+  </si>
+  <si>
+    <t xml:space="preserve">概要・詳細</t>
   </si>
   <si>
     <r>
@@ -2616,31 +2542,31 @@
     <t xml:space="preserve">Project setup</t>
   </si>
   <si>
-    <t xml:space="preserve">Khởi tạo project, kiến trúc phân tầng, cấu hình build</t>
+    <t xml:space="preserve">プロジェクト初期化・階層アーキテクチャ設計・ビルド構成</t>
   </si>
   <si>
     <t xml:space="preserve">Splash</t>
   </si>
   <si>
-    <t xml:space="preserve">Màn hình splash (logo, version)</t>
+    <t xml:space="preserve">スプラッシュ画面実装（企業ロゴ・バージョン表示）</t>
   </si>
   <si>
     <t xml:space="preserve">Start screen</t>
   </si>
   <si>
-    <t xml:space="preserve">Màn chọn receiver/transmitter + navigation</t>
+    <t xml:space="preserve">モード選択画面・ナビゲーション実装</t>
   </si>
   <si>
     <t xml:space="preserve">Permission</t>
   </si>
   <si>
-    <t xml:space="preserve">Xin quyền vị trí/BT/media/thông báo + dialog + thoát app</t>
+    <t xml:space="preserve">権限リクエストダイアログ（位置情報/BLE/通知）実装</t>
   </si>
   <si>
     <t xml:space="preserve">Common UI</t>
   </si>
   <si>
-    <t xml:space="preserve">Theme, asset, component thông báo/toast/dialog dùng chung</t>
+    <t xml:space="preserve">共通UIテーマ・トースト・ダイアログコンポーネント実装</t>
   </si>
   <si>
     <t xml:space="preserve">BLE Transport</t>
@@ -2649,49 +2575,49 @@
     <t xml:space="preserve">Central manager</t>
   </si>
   <si>
-    <t xml:space="preserve">CBCentralManager setup + quản lý state</t>
+    <t xml:space="preserve">Bluetooth Centralマネージャー初期化・状態管理</t>
   </si>
   <si>
     <t xml:space="preserve">Scan &amp; list</t>
   </si>
   <si>
-    <t xml:space="preserve">Quét + lọc (MPL R / MPL T) + danh sách thiết bị</t>
+    <t xml:space="preserve">デバイススキャン・フィルタリング・デバイス一覧表示</t>
   </si>
   <si>
     <t xml:space="preserve">Connect</t>
   </si>
   <si>
-    <t xml:space="preserve">Connect/disconnect/cancel/timeout 10s + thông điệp</t>
+    <t xml:space="preserve">接続・切断・タイムアウト制御・エラーメッセージ表示</t>
   </si>
   <si>
     <t xml:space="preserve">Auto reconnect</t>
   </si>
   <si>
-    <t xml:space="preserve">Tự kết nối thiết bị đã nhớ + tự reconnect</t>
+    <t xml:space="preserve">登録済みデバイス自動再接続ロジック実装</t>
   </si>
   <si>
     <t xml:space="preserve">RSSI</t>
   </si>
   <si>
-    <t xml:space="preserve">Giám sát RSSI + đổi màu trạng thái tín hiệu</t>
+    <t xml:space="preserve">RSSIシグナル監視・電波強度ステータスカラー反映</t>
   </si>
   <si>
     <t xml:space="preserve">GATT framing</t>
   </si>
   <si>
-    <t xml:space="preserve">Ghi/notify GATT + ghép gói (chunking) theo \r\n</t>
+    <t xml:space="preserve">GATTデータ送受信・パケットチャンキング処理</t>
   </si>
   <si>
     <t xml:space="preserve">Background BLE</t>
   </si>
   <si>
-    <t xml:space="preserve">Background mode + State Preservation/Restoration (rủi ro cao)</t>
+    <t xml:space="preserve">バックグラウンドモード・状態復元処理</t>
   </si>
   <si>
     <t xml:space="preserve">Protocol core</t>
   </si>
   <si>
-    <t xml:space="preserve">Encode/decode lệnh dùng chung</t>
+    <t xml:space="preserve">コマンドエンコード/デコード共通ライブラリ実装</t>
   </si>
   <si>
     <t xml:space="preserve">Receiver</t>
@@ -2700,141 +2626,85 @@
     <t xml:space="preserve">Main screen</t>
   </si>
   <si>
-    <t xml:space="preserve">Màn chính + UI/trạng thái kết nối</t>
+    <t xml:space="preserve">メイン画面UI・接続ステータスインジケーター</t>
   </si>
   <si>
     <t xml:space="preserve">Measurement recv</t>
   </si>
   <si>
-    <t xml:space="preserve">Nhận dữ liệu đo (parse *RMD, list, append)</t>
+    <t xml:space="preserve">測定データ受信パース・リスト追記処理</t>
   </si>
   <si>
     <t xml:space="preserve">Stored data download</t>
   </si>
   <si>
-    <t xml:space="preserve">Tải dữ liệu lưu (&amp;TMD, progress, abort)</t>
+    <t xml:space="preserve">保存データダウンロード・プログレスバー・中断処理</t>
   </si>
   <si>
     <t xml:space="preserve">Detail view</t>
   </si>
   <si>
-    <t xml:space="preserve">Xem chi tiết dữ liệu (swipe/tap)</t>
+    <t xml:space="preserve">測定詳細データ閲覧画面（スワイプ/タップ操作）</t>
   </si>
   <si>
     <t xml:space="preserve">Delete data</t>
   </si>
   <si>
-    <t xml:space="preserve">Xoá từng + xoá tất cả + dialog xác nhận</t>
+    <t xml:space="preserve">データ個別削除・一括削除・確認ダイアログ</t>
   </si>
   <si>
     <t xml:space="preserve">Log data create</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">Tạo </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="DejaVu Sans"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">現場データ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">: form, validation, 7 loại ống, check trùng tên</t>
-    </r>
+    <t xml:space="preserve">現場データ登録フォーム・バリデーション・重複チェック</t>
   </si>
   <si>
     <t xml:space="preserve">Log data list</t>
   </si>
   <si>
-    <t xml:space="preserve">Màn xem/danh sách log + xoá</t>
+    <t xml:space="preserve">ログ一覧画面・ログクリア機能</t>
   </si>
   <si>
     <t xml:space="preserve">Transmitter</t>
   </si>
   <si>
-    <t xml:space="preserve">Màn chính (nút tần số/output/điều chỉnh)</t>
+    <t xml:space="preserve">周波数・出力設定メインコントロールUI</t>
   </si>
   <si>
     <t xml:space="preserve">Remote control</t>
   </si>
   <si>
-    <t xml:space="preserve">Lệnh điều khiển + answerback (bảng 1/2/3)</t>
+    <t xml:space="preserve">制御コマンド送信・応答アンサーバリュー照合</t>
   </si>
   <si>
     <t xml:space="preserve">Current adjust</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">Điều chỉnh dòng (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="DejaVu Sans"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">直接法</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">) + nhãn giới hạn/max</t>
-    </r>
+    <t xml:space="preserve">電流直接調整制御・リミット上限表示</t>
   </si>
   <si>
     <t xml:space="preserve">Battery &amp; update</t>
   </si>
   <si>
-    <t xml:space="preserve">Hiển thị pin + cập nhật dữ liệu</t>
+    <t xml:space="preserve">バッテリー残量表示・定期ポーリング更新</t>
   </si>
   <si>
     <t xml:space="preserve">Sleep</t>
   </si>
   <si>
-    <t xml:space="preserve">Chức năng sleep (dialog, trạng thái)</t>
+    <t xml:space="preserve">スリープモード移行・ステータスダイアログ</t>
   </si>
   <si>
     <t xml:space="preserve">Background op</t>
   </si>
   <si>
-    <t xml:space="preserve">Duy trì kết nối nền (riêng TX) + ánh xạ thông báo</t>
+    <t xml:space="preserve">送信機バックグラウンドキープアライブ制御</t>
   </si>
   <si>
     <t xml:space="preserve">Error handling</t>
   </si>
   <si>
-    <t xml:space="preserve">Xử lý timeout 3s + gửi lại x2</t>
+    <t xml:space="preserve">3秒タイムアウト制御・最大2回リトライ処理</t>
   </si>
   <si>
     <t xml:space="preserve">GPS</t>
@@ -2843,19 +2713,19 @@
     <t xml:space="preserve">Internal GPS</t>
   </si>
   <si>
-    <t xml:space="preserve">GPS nội bộ (Core Location) + UI chuyển nguồn</t>
+    <t xml:space="preserve">内部GPS測位連携・測位ソース切替UI</t>
   </si>
   <si>
     <t xml:space="preserve">External GPS</t>
   </si>
   <si>
-    <t xml:space="preserve">GPS ngoài (Geode/BLE): connect/chọn/pin/disconnect (rủi ro cao)</t>
+    <t xml:space="preserve">外部GPSレシーバー連携・BLE接続管理</t>
   </si>
   <si>
     <t xml:space="preserve">GPS binding</t>
   </si>
   <si>
-    <t xml:space="preserve">Gắn dữ liệu GPS vào dữ liệu đo (lat/long/sai số/độ cao)</t>
+    <t xml:space="preserve">GPS座標（緯度/経度/高度/誤差）メタデータ付与</t>
   </si>
   <si>
     <t xml:space="preserve">Map</t>
@@ -2864,19 +2734,19 @@
     <t xml:space="preserve">Map setup</t>
   </si>
   <si>
-    <t xml:space="preserve">Cấu hình map SDK (Google Maps iOS / MapKit) + key</t>
+    <t xml:space="preserve">地図SDK構成設定・APIキー認証組み込み</t>
   </si>
   <si>
     <t xml:space="preserve">Marker &amp; line</t>
   </si>
   <si>
-    <t xml:space="preserve">Marker + màu theo loại ống + nối line</t>
+    <t xml:space="preserve">マップマーカー描画・属性別カラーライン描画</t>
   </si>
   <si>
     <t xml:space="preserve">Location feature</t>
   </si>
   <si>
-    <t xml:space="preserve">Vị trí hiện tại/recenter/realtime/popup chi tiết</t>
+    <t xml:space="preserve">現在位置追従・リセンター・詳細ポップアップ表示</t>
   </si>
   <si>
     <t xml:space="preserve">File Export</t>
@@ -2885,19 +2755,19 @@
     <t xml:space="preserve">KML export</t>
   </si>
   <si>
-    <t xml:space="preserve">Sinh KML + màu/line + chia sẻ</t>
+    <t xml:space="preserve">KML地理空間データ生成・共有機能</t>
   </si>
   <si>
     <t xml:space="preserve">CSV export</t>
   </si>
   <si>
-    <t xml:space="preserve">Sinh CSV (cột theo spec) + chia sẻ</t>
+    <t xml:space="preserve">CSVエクスポート・ファイル共有連携</t>
   </si>
   <si>
     <t xml:space="preserve">Share sheet</t>
   </si>
   <si>
-    <t xml:space="preserve">Tích hợp share sheet + dialog lỗi</t>
+    <t xml:space="preserve">OS標準シェアシート連携・エラーダイアログ</t>
   </si>
   <si>
     <t xml:space="preserve">Storage &amp; Notification</t>
@@ -2906,13 +2776,13 @@
     <t xml:space="preserve">Local storage</t>
   </si>
   <si>
-    <t xml:space="preserve">Mô hình dữ liệu + persistence + giới hạn dung lượng</t>
+    <t xml:space="preserve">データ永続化モデリング・ローカルストレージ容量制御</t>
   </si>
   <si>
     <t xml:space="preserve">Notification</t>
   </si>
   <si>
-    <t xml:space="preserve">Local notification (trạng thái TX) + chỉ báo foreground</t>
+    <t xml:space="preserve">ローカルプッシュ通知・フォアグラウンドインジケーター</t>
   </si>
   <si>
     <t xml:space="preserve">小計</t>
@@ -2939,72 +2809,16 @@
     <t xml:space="preserve">完成図書</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">Lập tài liệu hoàn công: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="DejaVu Sans"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">構成図</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="DejaVu Sans"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">パラメータ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="DejaVu Sans"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">試験結果</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Tiếng Nhật, mức chi tiết tiêu chuẩn</t>
+    <t xml:space="preserve">納品ドキュメント作成（システム構成図、各種パラメータ設定書、試験結果報告書）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">日本語、標準詳細度</t>
   </si>
   <si>
     <t xml:space="preserve">Handover</t>
   </si>
   <si>
-    <t xml:space="preserve">Bàn giao &amp; giải thích tài liệu</t>
+    <t xml:space="preserve">運用引継ぎおよび各種設計・手順ドキュメントの説明・質疑応答</t>
   </si>
   <si>
     <t xml:space="preserve">結合テスト</t>
@@ -3013,91 +2827,16 @@
     <t xml:space="preserve">Test design</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">Lập test plan &amp; test case (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="DejaVu Sans"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">単体 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="DejaVu Sans"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">結合</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">テスト計画書・テストケース作成（単体テスト・結合テスト仕様）</t>
   </si>
   <si>
     <t xml:space="preserve">Integration test</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">Kịch bản end-to-end: web</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="DejaVu Sans"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">会議 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Meiryo UI"/>
-        <family val="2"/>
-        <charset val="128"/>
-      </rPr>
-      <t xml:space="preserve">thông, luồng khác bị chặn</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">Môi trường test sẵn sàng</t>
+    <t xml:space="preserve">エンドツーエンド結合テストシナリオ検証・不具合修正</t>
+  </si>
+  <si>
+    <t xml:space="preserve">テスト検証環境提供前提</t>
   </si>
   <si>
     <r>
@@ -4842,46 +4581,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>276120</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>95400</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>171720</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>217080</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="image1.png" descr="rikkei.png"/>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch/>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6749280" y="95400"/>
-          <a:ext cx="1969560" cy="1055160"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="0">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5096,7 +4796,7 @@
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="7" name="Mũi tên phải 1"/>
+        <xdr:cNvPr id="7" name="Mũi tn phải 1"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -5149,7 +4849,7 @@
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="8" name="Mũi tên phải 2"/>
+        <xdr:cNvPr id="8" name="Mũi tn phải 2"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -5202,7 +4902,7 @@
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="9" name="Mũi tên phải 3"/>
+        <xdr:cNvPr id="9" name="Mũi tn phải 3"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -5255,7 +4955,7 @@
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="10" name="Mũi tên phải 4"/>
+        <xdr:cNvPr id="10" name="Mũi tn phải 4"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -5308,7 +5008,7 @@
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="11" name="Mũi tên phải 6"/>
+        <xdr:cNvPr id="11" name="Mũi tn phải 6"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -5361,7 +5061,7 @@
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="12" name="Mũi tên phải 8"/>
+        <xdr:cNvPr id="12" name="Mũi tn phải 8"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -5414,7 +5114,7 @@
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
-        <xdr:cNvPr id="13" name="Mũi tên phải 9"/>
+        <xdr:cNvPr id="13" name="Mũi tn phải 9"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -5472,7 +5172,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="image7.png" descr="rikkei.png"/>
+        <xdr:cNvPr id="14" name="image7.png" descr="development team.png"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -5515,7 +5215,7 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="15" name="image11.png" descr="rikkei.png"/>
+        <xdr:cNvPr id="15" name="image11.png" descr="development team.png"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -9516,7 +9216,7 @@
     <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="167" t="str">
         <f aca="false">表紙!B14</f>
-        <v>MPL-H12 App_IOS</v>
+        <v>法人向け契約・請求・入金管理システム</v>
       </c>
       <c r="C11" s="167"/>
       <c r="D11" s="167"/>
@@ -9905,7 +9605,7 @@
     <row r="9" customFormat="false" ht="56.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="188" t="str">
         <f aca="false">表紙!B14</f>
-        <v>MPL-H12 App_IOS</v>
+        <v>法人向け契約・請求・入金管理システム</v>
       </c>
       <c r="B9" s="188"/>
       <c r="C9" s="188"/>

</xml_diff>